<commit_message>
Enhance auto-reply functionality with a detailed HTML template and add new inquiry entries to data files
</commit_message>
<xml_diff>
--- a/data/inquiries.xlsx
+++ b/data/inquiries.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,6 +682,240 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>sales5@araspl.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Flat, Plate, Steel Product</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlni0AAA=</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-09-09T06:45:47.113696+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>roybishal200189@gmail.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Plate, Flat, Steel Product</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjIAAA=</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-10T06:10:23.438824+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>roybishal200189@gmail.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Angle</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjHAAA=</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-09-10T06:10:24.052965+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>roybishal200189@gmail.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Steel Product, Flat, Plate</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjLAAA=</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-09-10T06:19:08.389742+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>roybishal200189@gmail.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Steel Product, Plate, Flat</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjMAAA=</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-09-10T06:53:00.139420+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>roybishal200189@gmail.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Plate, Steel Product, Flat</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjNAAA=</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-09-10T06:55:43.575912+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>hr1@araspl.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Plate, Flat, Angle</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjPAAA=</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-09-10T08:11:58.673291+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>roybishal200189@gmail.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Plate, Flat, Steel Product</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjRAAA=</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-10T12:24:28.584875+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>roybishal200189@gmail.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Plate, Flat, Steel Product</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>AAMkADM0OWM2NTdkLWRlZWEtNDlkMS05ZWQyLTQyZDZkYjc5YmQ5OQBGAAAAAABlGtqsIfsRQJ2u_5ZGJ3n0BwBJQ8M0YfOHQJCBZSJHT0p_AAAAAAEMAABJQ8M0YfOHQJCBZSJHT0p_AAFKlnjSAAA=</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-09-10T12:34:52.973215+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>